<commit_message>
chore: daily swing scan and journal refresh
</commit_message>
<xml_diff>
--- a/reports/swing_performance.xlsx
+++ b/reports/swing_performance.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Picks" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Runs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Picks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Picks'!$A$1:$Z$18</definedName>
@@ -759,7 +759,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>TARGET1_HIT</t>
+          <t>TARGET2_HIT</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -772,17 +772,31 @@
           <t>2026-08-06</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>1878.24</v>
+      </c>
+      <c r="V3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1.3</v>
+      </c>
       <c r="X3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Backfilled from manual scan</t>
+          <t>Assumes 50% booked at T1 and 50% at T2</t>
         </is>
       </c>
     </row>
@@ -943,7 +957,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>TIME_EXIT</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -951,17 +965,32 @@
           <t>2026-08-06</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>1369</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.05</v>
+      </c>
       <c r="X5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Backfilled from 2026-08-06 manual scan</t>
+          <t>Closed after 10 sessions</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1059,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>STOPPED</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1038,17 +1067,32 @@
           <t>2026-08-06</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>1857.63</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-4.25</v>
+      </c>
+      <c r="W6" t="n">
+        <v>-1</v>
+      </c>
       <c r="X6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>nearest support + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Structural stop hit</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1363,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>TARGET1_HIT</t>
+          <t>BREAKEVEN_AFTER_T1</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1332,17 +1376,31 @@
           <t>2026-08-14</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>35.91</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.5</v>
+      </c>
       <c r="X9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>nearest support + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Second half stopped at cost after T1</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1787,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>TIME_EXIT</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1737,17 +1795,32 @@
           <t>2026-08-11</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>853.45</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.15</v>
+      </c>
       <c r="X13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>nearest resistance + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Closed after 10 sessions</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1889,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>TIME_EXIT</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1824,17 +1897,32 @@
           <t>2026-08-12</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>489.55</v>
+      </c>
+      <c r="V14" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.55</v>
+      </c>
       <c r="X14" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>nearest support + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Closed after 10 sessions</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1991,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>STOPPED</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1911,17 +1999,32 @@
           <t>2026-08-12</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>1659.26</v>
+      </c>
+      <c r="V15" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="W15" t="n">
+        <v>-1</v>
+      </c>
       <c r="X15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>nearest support + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Structural stop hit</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2194,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>STOPPED</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2099,17 +2202,32 @@
           <t>2026-08-13</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>512.84</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="W17" t="n">
+        <v>-1</v>
+      </c>
       <c r="X17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>nearest support + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Structural stop hit</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2296,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>TIME_EXIT</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2186,17 +2304,36 @@
           <t>2026-08-14</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>183.49</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="W18" t="n">
+        <v>1.15</v>
+      </c>
       <c r="X18" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>nearest resistance + ATR buffer; target at ATR projection; hold 5-10 trading days</t>
+          <t>Closed after 10 sessions</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2752,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-17T16:05:17</t>
+          <t>2026-08-28T22:32:30</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2773,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2646,7 +2783,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -2656,7 +2793,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -2666,7 +2803,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -2676,7 +2813,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>58.82</v>
       </c>
     </row>
     <row r="9">
@@ -2686,7 +2823,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.05</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="10">
@@ -2696,7 +2833,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2706,7 +2843,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.43</v>
+        <v>3.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: daily swing scan, journal and history refresh
</commit_message>
<xml_diff>
--- a/reports/swing_performance.xlsx
+++ b/reports/swing_performance.xlsx
@@ -965,7 +965,6 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>2026-08-19</t>
@@ -1067,7 +1066,6 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>2026-08-19</t>
@@ -1795,7 +1793,6 @@
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>2026-08-24</t>
@@ -1897,7 +1894,6 @@
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>2026-08-25</t>
@@ -1999,7 +1995,6 @@
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>2026-08-18</t>
@@ -2202,7 +2197,6 @@
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>2026-08-19</t>
@@ -2752,7 +2746,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28T22:32:30</t>
+          <t>2026-08-31T19:14:07</t>
         </is>
       </c>
     </row>

</xml_diff>